<commit_message>
Fix table field names exceeding the 16-char DB field limit
LOGICAL_STATUS_CODE (19) -> STATUS_CODE, MBLNR_HANDLED_MANUALLY (22)
-> MBLNR_MANUAL. SE11 silently truncates longer names. Program aliases
and both setup Excels updated to match.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DJGnX3fs4N1zpoFwvs7VjS
</commit_message>
<xml_diff>
--- a/src/abap/snapshot/_setup_ILG_MM_GP_SNAP.xlsx
+++ b/src/abap/snapshot/_setup_ILG_MM_GP_SNAP.xlsx
@@ -449,6 +449,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -543,10 +544,9 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LOGICAL_STATUS_CODE</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>STATUS_CODE</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>CHAR2</t>
@@ -570,7 +570,6 @@
           <t>LOGICAL_STATUS</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>CHAR40</t>
@@ -594,7 +593,6 @@
           <t>IS_MONITOR</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>CHAR1</t>
@@ -618,7 +616,6 @@
           <t>MBLNR</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>MBLNR</t>
@@ -639,10 +636,9 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MBLNR_HANDLED_MANUALLY</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
+          <t>MBLNR_MANUAL</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>CHAR1</t>
@@ -666,7 +662,6 @@
           <t>BELNR_MM</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>RE_BELNR</t>
@@ -690,7 +685,6 @@
           <t>GJAHR_MM</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>GJAHR</t>
@@ -714,7 +708,6 @@
           <t>RBSTAT</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>RBSTAT</t>
@@ -738,7 +731,6 @@
           <t>BUKRS</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>BUKRS</t>
@@ -762,7 +754,6 @@
           <t>BELNR_FI</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>BELNR_D</t>
@@ -786,7 +777,6 @@
           <t>GJAHR_FI</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>GJAHR</t>
@@ -810,7 +800,6 @@
           <t>IS_PAID</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>CHAR1</t>
@@ -834,7 +823,6 @@
           <t>AUGBL</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>AUGBL</t>
@@ -858,7 +846,6 @@
           <t>AUGDT</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>AUGDT</t>
@@ -882,7 +869,6 @@
           <t>IS_REVERSED</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
           <t>CHAR1</t>
@@ -906,7 +892,6 @@
           <t>STGRD</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>STGRD</t>
@@ -930,7 +915,6 @@
           <t>STGRD_TXT</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>TXT40</t>
@@ -954,7 +938,6 @@
           <t>AEDAT</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>AEDAT</t>
@@ -978,7 +961,6 @@
           <t>AEZET</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>AEZET</t>

</xml_diff>